<commit_message>
Some updates of reports
</commit_message>
<xml_diff>
--- a/ProjectReports/Gant Table.xlsx
+++ b/ProjectReports/Gant Table.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{2566B9CB-C597-4B75-8D11-821E0E8CA690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6278F261-76AB-41C0-A385-933E7EBB5E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -885,6 +885,9 @@
     <xf numFmtId="178" fontId="27" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -902,9 +905,6 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="10" applyFont="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1397,60 +1397,60 @@
         <v>1</v>
       </c>
       <c r="J2" s="8"/>
-      <c r="K2" s="27"/>
+      <c r="K2" s="21"/>
       <c r="L2" s="28"/>
       <c r="M2" s="29"/>
       <c r="N2" s="9"/>
-      <c r="O2" s="27" t="s">
+      <c r="O2" s="21" t="s">
         <v>6</v>
       </c>
       <c r="P2" s="28"/>
       <c r="Q2" s="28"/>
       <c r="R2" s="29"/>
       <c r="S2" s="10"/>
-      <c r="T2" s="27" t="s">
+      <c r="T2" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
       <c r="W2" s="30"/>
       <c r="X2" s="11"/>
-      <c r="Y2" s="27" t="s">
+      <c r="Y2" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="21"/>
-      <c r="AA2" s="21"/>
-      <c r="AB2" s="21"/>
+      <c r="Z2" s="22"/>
+      <c r="AA2" s="22"/>
+      <c r="AB2" s="22"/>
       <c r="AC2" s="30"/>
       <c r="AD2" s="12"/>
-      <c r="AE2" s="27" t="s">
+      <c r="AE2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="AF2" s="21"/>
-      <c r="AG2" s="21"/>
-      <c r="AH2" s="21"/>
-      <c r="AI2" s="21"/>
-      <c r="AJ2" s="21"/>
-      <c r="AK2" s="21"/>
-      <c r="AL2" s="21"/>
+      <c r="AF2" s="22"/>
+      <c r="AG2" s="22"/>
+      <c r="AH2" s="22"/>
+      <c r="AI2" s="22"/>
+      <c r="AJ2" s="22"/>
+      <c r="AK2" s="22"/>
+      <c r="AL2" s="22"/>
     </row>
     <row r="3" spans="2:67" s="16" customFormat="1" ht="39.950000000000003" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="27" t="s">
         <v>3</v>
       </c>
       <c r="H3" s="13" t="s">
@@ -1477,12 +1477,12 @@
       <c r="AA3" s="15"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="23"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="20">
         <v>1</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>6</v>
       </c>
       <c r="G6" s="19">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
@@ -1721,7 +1721,7 @@
         <v>5</v>
       </c>
       <c r="G7" s="19">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8" spans="2:67" ht="43.5" customHeight="1" x14ac:dyDescent="0.4">
@@ -1741,7 +1741,7 @@
         <v>6</v>
       </c>
       <c r="G8" s="19">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9" spans="2:67" ht="45.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1761,7 +1761,7 @@
         <v>2</v>
       </c>
       <c r="G9" s="19">
-        <v>0.4</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
@@ -1801,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="19">
-        <v>0</v>
+        <v>0.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>